<commit_message>
Adjust scripts 1 and 2: - set cycles to 0 for state before (script 1) - change cut-offs for NMP_cat (script 1) - compute stats based on Sediment (script 2)
</commit_message>
<xml_diff>
--- a/analysis/derived_data/FT_STA_formatted-data.xlsx
+++ b/analysis/derived_data/FT_STA_formatted-data.xlsx
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="C2">
-        <v>276</v>
+        <v>600</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="C3">
-        <v>276</v>
+        <v>600</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -844,7 +844,7 @@
         </is>
       </c>
       <c r="C4">
-        <v>276</v>
+        <v>600</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -979,7 +979,7 @@
         </is>
       </c>
       <c r="C5">
-        <v>276</v>
+        <v>600</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="C6">
-        <v>276</v>
+        <v>0</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="C7">
-        <v>276</v>
+        <v>0</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="C8">
-        <v>276</v>
+        <v>0</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="C9">
-        <v>276</v>
+        <v>0</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -2194,7 +2194,7 @@
         </is>
       </c>
       <c r="C14">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -2329,7 +2329,7 @@
         </is>
       </c>
       <c r="C15">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -2464,7 +2464,7 @@
         </is>
       </c>
       <c r="C16">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -2599,7 +2599,7 @@
         </is>
       </c>
       <c r="C17">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -3274,7 +3274,7 @@
         </is>
       </c>
       <c r="C22">
-        <v>476</v>
+        <v>0</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -3409,7 +3409,7 @@
         </is>
       </c>
       <c r="C23">
-        <v>476</v>
+        <v>0</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -3544,7 +3544,7 @@
         </is>
       </c>
       <c r="C24">
-        <v>476</v>
+        <v>0</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -3679,7 +3679,7 @@
         </is>
       </c>
       <c r="C25">
-        <v>476</v>
+        <v>0</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="C30">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -4489,7 +4489,7 @@
         </is>
       </c>
       <c r="C31">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -4624,7 +4624,7 @@
         </is>
       </c>
       <c r="C32">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -4759,7 +4759,7 @@
         </is>
       </c>
       <c r="C33">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -5434,7 +5434,7 @@
         </is>
       </c>
       <c r="C38">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -5569,7 +5569,7 @@
         </is>
       </c>
       <c r="C39">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -5704,7 +5704,7 @@
         </is>
       </c>
       <c r="C40">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -5839,7 +5839,7 @@
         </is>
       </c>
       <c r="C41">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -6514,7 +6514,7 @@
         </is>
       </c>
       <c r="C46">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -6649,7 +6649,7 @@
         </is>
       </c>
       <c r="C47">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -6784,7 +6784,7 @@
         </is>
       </c>
       <c r="C48">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -6919,7 +6919,7 @@
         </is>
       </c>
       <c r="C49">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -7594,7 +7594,7 @@
         </is>
       </c>
       <c r="C54">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -7729,7 +7729,7 @@
         </is>
       </c>
       <c r="C55">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -7864,7 +7864,7 @@
         </is>
       </c>
       <c r="C56">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -7999,7 +7999,7 @@
         </is>
       </c>
       <c r="C57">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -8674,7 +8674,7 @@
         </is>
       </c>
       <c r="C62">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -8809,7 +8809,7 @@
         </is>
       </c>
       <c r="C63">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -8944,7 +8944,7 @@
         </is>
       </c>
       <c r="C64">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -9079,7 +9079,7 @@
         </is>
       </c>
       <c r="C65">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -9754,7 +9754,7 @@
         </is>
       </c>
       <c r="C70">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -9889,7 +9889,7 @@
         </is>
       </c>
       <c r="C71">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -10024,7 +10024,7 @@
         </is>
       </c>
       <c r="C72">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -10159,7 +10159,7 @@
         </is>
       </c>
       <c r="C73">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -10834,7 +10834,7 @@
         </is>
       </c>
       <c r="C78">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -10969,7 +10969,7 @@
         </is>
       </c>
       <c r="C79">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -11104,7 +11104,7 @@
         </is>
       </c>
       <c r="C80">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -11239,7 +11239,7 @@
         </is>
       </c>
       <c r="C81">
-        <v>330</v>
+        <v>0</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>

</xml_diff>